<commit_message>
fix import upload path, ledger ordering and misleading UI states
Uploads never reached S3: the CloudFront CSP omitted the import bucket and
the presigned URL used SigV2 against the global endpoint, which 307-redirects
regional buckets. Jobs then sat in awaiting_upload forever with no expiry.

Ledger pages were keyed by random transaction id, so the audit trail could not
be browsed chronologically; existing rows were migrated to a time-based key.

Also fixes a replenishment receipt replaying an earlier overage as a new one,
adds the adjustment reason to the ledger, keeps rejected requests from locking
the operation forms, and guards against deploying a stale lambda package.
</commit_message>
<xml_diff>
--- a/fixtures/purchase-order-sample.xlsx
+++ b/fixtures/purchase-order-sample.xlsx
@@ -1,13 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
-    <sheet name="採購單匯入範例" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="purchase_orders" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'採購單匯入範例'!$A$1:$G$9</definedName>
-  </definedNames>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -410,16 +413,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -462,31 +465,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PO-20260918-001</t>
+          <t>PO-TEST-100</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>??????</t>
+          <t>匯入測試供應商</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MAT-IC-2001</t>
+          <t>MAT-5001</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>??????</t>
+          <t>墊片</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>240</v>
+        <v>30</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -497,31 +500,31 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PO-20260918-001</t>
+          <t>PO-TEST-100</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>??????</t>
+          <t>匯入測試供應商</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MAT-CAP-1102</t>
+          <t>MAT-5002</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>?????</t>
+          <t>軸心</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>120</v>
+        <v>15</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -532,215 +535,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PO-20260922-002</t>
+          <t>PO-TEST-101</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>??????</t>
+          <t>匯入測試供應商</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MAT-STEEL-3001</t>
+          <t>MAT-5003</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>??????</t>
+          <t>彈簧</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>pcs</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>PO-20260922-002</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>??????</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>MAT-BOLT-3002</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>M8 ????</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>600</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>PO-20260925-003</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>????????</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>MAT-BOX-4101</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>???? S</t>
-        </is>
-      </c>
-      <c r="F6" t="n">
-        <v>500</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>PO-20260925-003</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>????????</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>MAT-TAPE-4102</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>????</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>60</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>PO-20260930-004</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>??????</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>MAT-LABEL-5201</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>?????</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>100</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>PO-20260930-004</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>??????</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>MAT-RIBBON-5202</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>????</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>40</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>?</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>